<commit_message>
Excel Practice @ Day 08 to 10
</commit_message>
<xml_diff>
--- a/Excel Practice @ Day 01.xlsx
+++ b/Excel Practice @ Day 01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Codegnan\Data Analytics\Microsoft Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MY FILES\M S Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A226BE5D-83E1-4910-85CC-6E7D0D6E789C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F8B54E3-F3C1-4E0F-B0FA-A05B41AFF93F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5FB56502-8CCC-4FEF-933B-4B92691D64CD}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{5FB56502-8CCC-4FEF-933B-4B92691D64CD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -445,12 +445,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{434D2FB2-2A93-4150-8783-1D0D51BE71F1}">
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="5" max="5" width="17.77734375" customWidth="1"/>
+    <col min="5" max="5" width="17.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -467,7 +467,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
         <v>4</v>
       </c>
@@ -480,7 +480,7 @@
       <c r="D2" s="5"/>
       <c r="E2" s="6"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>5</v>
       </c>
@@ -493,7 +493,7 @@
       <c r="D3" s="5"/>
       <c r="E3" s="6"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>6</v>
       </c>
@@ -506,7 +506,7 @@
       <c r="D4" s="5"/>
       <c r="E4" s="6"/>
     </row>
-    <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
@@ -520,7 +520,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
         <v>4</v>
       </c>
@@ -530,9 +530,12 @@
       <c r="C8" s="7">
         <v>0.1</v>
       </c>
-      <c r="D8" s="5"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D8">
+        <f>B8*C8</f>
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>5</v>
       </c>
@@ -542,9 +545,12 @@
       <c r="C9" s="7">
         <v>0.1</v>
       </c>
-      <c r="D9" s="5"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D9">
+        <f t="shared" ref="D9:D10" si="0">B9*C9</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
         <v>6</v>
       </c>
@@ -554,19 +560,22 @@
       <c r="C10" s="7">
         <v>0.1</v>
       </c>
-      <c r="D10" s="5"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D10">
+        <f t="shared" si="0"/>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B12" s="2"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B15" s="1"/>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B16">
         <v>1</v>
       </c>
@@ -583,55 +592,130 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="4">
         <v>1</v>
       </c>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B17" s="2">
+        <f>$A17*B$16</f>
+        <v>1</v>
+      </c>
+      <c r="C17" s="2">
+        <f t="shared" ref="C17:F17" si="1">$A17*C$16</f>
+        <v>2</v>
+      </c>
+      <c r="D17" s="2">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="E17" s="2">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="F17" s="2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="4">
         <v>2</v>
       </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B18" s="2">
+        <f t="shared" ref="B18:F21" si="2">$A18*B$16</f>
+        <v>2</v>
+      </c>
+      <c r="C18" s="2">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="D18" s="2">
+        <f t="shared" si="2"/>
+        <v>6</v>
+      </c>
+      <c r="E18" s="2">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="F18" s="2">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="4">
         <v>3</v>
       </c>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B19" s="2">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="C19" s="2">
+        <f t="shared" si="2"/>
+        <v>6</v>
+      </c>
+      <c r="D19" s="2">
+        <f t="shared" si="2"/>
+        <v>9</v>
+      </c>
+      <c r="E19" s="2">
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="F19" s="2">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="4">
         <v>4</v>
       </c>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B20" s="2">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="C20" s="2">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="D20" s="2">
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="E20" s="2">
+        <f t="shared" si="2"/>
+        <v>16</v>
+      </c>
+      <c r="F20" s="2">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="4">
         <v>5</v>
       </c>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
+      <c r="B21" s="2">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="C21" s="2">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="D21" s="2">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+      <c r="E21" s="2">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="F21" s="2">
+        <f t="shared" si="2"/>
+        <v>25</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>